<commit_message>
readme: added built features
</commit_message>
<xml_diff>
--- a/Platform_SRS_file/tables/Appendices.xlsx
+++ b/Platform_SRS_file/tables/Appendices.xlsx
@@ -5,7 +5,7 @@
   <workbookPr filterPrivacy="1"/>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{77893F20-99C3-4808-AC41-389593B82C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23260" windowHeight="15280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Traceability Table, Section 9.1" sheetId="4" r:id="rId1"/>
@@ -1252,13 +1252,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1326,10 +1326,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2569,7 +2565,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H3:H12 I20 I22 H14:H18 H20:H28">
+  <conditionalFormatting sqref="H3:H12 H14:H18 I20 H20:H28 I22">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="notEqual">
       <formula>"Built"</formula>
     </cfRule>
@@ -3078,6 +3074,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010072A6C8471E7210488FB2A8F69895B9CC" ma:contentTypeVersion="1" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="76e91a76b45ea764b42bbb1898e61559">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="29671bd3-f04c-44c5-994c-1a02d2686427" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8721d2c1d2406d62ed386112b33a31a7" ns3:_="">
     <xsd:import namespace="29671bd3-f04c-44c5-994c-1a02d2686427"/>
@@ -3203,22 +3214,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1B6F82E0-B02C-4B05-AF5A-BA362433C7EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="29671bd3-f04c-44c5-994c-1a02d2686427"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FDD99FC-CBE6-412D-9919-A21CCB41123E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B0B01405-9A5B-4AA5-BA93-BF30C137752D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3234,28 +3254,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FDD99FC-CBE6-412D-9919-A21CCB41123E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1B6F82E0-B02C-4B05-AF5A-BA362433C7EA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="29671bd3-f04c-44c5-994c-1a02d2686427"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>